<commit_message>
Prepare audience-facing lecture materials and remove internal reviews
</commit_message>
<xml_diff>
--- a/demo-runs/2026-10-17/demo3_dcf_valuation/GOOGL_DCF_Valuation.xlsx
+++ b/demo-runs/2026-10-17/demo3_dcf_valuation/GOOGL_DCF_Valuation.xlsx
@@ -90,7 +90,7 @@
     <t>Forward P/E uses CY2027 adjusted consensus EPS dated Oct 16. Microsoft is calendarized from FY2027 / FY2028.</t>
   </si>
   <si>
-    <t>Teaching model, not investment advice. Market and scenario assumptions require presenter review.</t>
+    <t>Teaching model, not investment advice. Market and scenario assumptions are dated and uncertain.</t>
   </si>
   <si>
     <t>Sources (IDs also appear beside the inputs)</t>
@@ -180,7 +180,7 @@
     <t>https://www.google.com/finance/quote/AMZN:NASDAQ</t>
   </si>
   <si>
-    <t>A1 — Author teaching assumptions, October 17, 2026; not company guidance</t>
+    <t>A1 — Teaching assumptions, October 17, 2026; not company guidance</t>
   </si>
   <si>
     <t>valuation-notes.md</t>
@@ -1227,7 +1227,7 @@
     <t>No SBC, content, operating-lease asset or other cash-flow addbacks. EV excludes lease liabilities uniformly; lease mixes still differ.</t>
   </si>
   <si>
-    <t>Full TTM intangible amortization is not verified for GOOGL / AMZN. EBITD replaces EBITDA by the presenter’s choice; it is not EBITDA.</t>
+    <t>Full TTM intangible amortization is unavailable for GOOGL / AMZN. EBITD adds PP&amp;E depreciation; intangible amortization stays expensed.</t>
   </si>
 </sst>
 </file>

</xml_diff>